<commit_message>
test(xlsx): sample phủ 10 quy tắc + nhãn inline, verify khớp output
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/xlsx-bad.xlsx
+++ b/samples/xlsx-bad.xlsx
@@ -27,12 +27,17 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -47,8 +52,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -123,6 +129,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>pm</author>
+  </authors>
+  <commentList>
+    <comment ref="B4" authorId="0" shapeId="0">
+      <text>
+        <t>Vượt kế hoạch 10% [vi phạm XLSX-05: chỉ trong comment]</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -414,13 +435,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>BÁO CÁO DOANH THU NĂM 2026</t>
+          <t>BÁO CÁO DOANH THU NĂM 2026 [vi phạm XLSX-01/02]</t>
         </is>
       </c>
     </row>
@@ -447,7 +468,7 @@
           <t>01</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="1" t="n">
         <v>110</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -474,11 +495,41 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Chi phí [vi phạm XLSX-10: bảng con thứ 2 chung sheet]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Khoản</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Số tiền</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -494,7 +545,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>dữ liệu nháp không nên lộ ra</t>
+          <t>dữ liệu nháp không nên lộ ra [vi phạm XLSX-06: sheet ẩn]</t>
         </is>
       </c>
     </row>

</xml_diff>